<commit_message>
Preserve original Excel style metadata and compatibility declarations
</commit_message>
<xml_diff>
--- a/20261020_170147_A3_LD_6Scenarios/A3_LD_가공SW_6시나리오_통합평가.xlsx
+++ b/20261020_170147_A3_LD_6Scenarios/A3_LD_가공SW_6시나리오_통합평가.xlsx
@@ -999,262 +999,262 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<s:styleSheet xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <s:fonts count="16">
-    <s:font>
-      <s:sz val="11"/>
-      <s:name val="Carlito"/>
-    </s:font>
-    <s:font>
-      <s:sz val="11"/>
-      <s:color rgb="FF1C344B"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:b/>
-      <s:sz val="16"/>
-      <s:color rgb="FF1C344B"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:b/>
-      <s:sz val="11"/>
-      <s:color rgb="FF1C344B"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:b/>
-      <s:sz val="11"/>
-      <s:color rgb="FF98510C"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:sz val="9"/>
-      <s:color rgb="FF536B7C"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:b/>
-      <s:sz val="11"/>
-      <s:color rgb="FFFFFFFF"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:sz val="11"/>
-      <s:color rgb="FF174E8C"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:sz val="9"/>
-      <s:color rgb="FF1C344B"/>
-      <s:name val="Malgun Gothic"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
-      <s:sz val="11"/>
-      <s:name val="Carlito"/>
-    </s:font>
-    <s:font>
-      <s:sz val="8"/>
-      <s:name val="돋움"/>
-      <s:family val="3"/>
-      <s:charset val="129"/>
-    </s:font>
-    <s:font>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="16">
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1C344B"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1C344B"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1C344B"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF98510C"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF536B7C"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF174E8C"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1C344B"/>
+      <name val="Malgun Gothic"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <s:font xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:sz val="11"/>
       <s:color rgb="FF1C344B"/>
       <s:name val="Malgun Gothic"/>
     </s:font>
-    <s:font>
+    <s:font xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:b/>
       <s:sz val="16"/>
       <s:color rgb="FF1C344B"/>
       <s:name val="Malgun Gothic"/>
     </s:font>
-    <s:font>
+    <s:font xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:sz val="11"/>
       <s:color rgb="FF536B7C"/>
       <s:name val="Malgun Gothic"/>
     </s:font>
-    <s:font>
+    <s:font xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:b/>
       <s:sz val="11"/>
       <s:color rgb="FFFFFFFF"/>
       <s:name val="Malgun Gothic"/>
     </s:font>
-    <s:font>
+    <s:font xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:b/>
       <s:sz val="11"/>
       <s:color rgb="FF1C344B"/>
       <s:name val="Malgun Gothic"/>
     </s:font>
-  </s:fonts>
-  <s:fills count="19">
-    <s:fill>
-      <s:patternFill patternType="none"/>
+  </fonts>
+  <fills count="19">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF244F7A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF244F7A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF244F7A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F1FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF244F7A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE5F4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <s:fill xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+      <s:patternFill patternType="solid">
+        <s:fgColor rgb="FFFFF7DE"/>
+      </s:patternFill>
     </s:fill>
-    <s:fill>
-      <s:patternFill patternType="gray125"/>
-    </s:fill>
-    <s:fill>
+    <s:fill xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:patternFill patternType="solid">
         <s:fgColor rgb="FF244F7A"/>
       </s:patternFill>
     </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF1D9"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF7DF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFFFFF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FF244F7A"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF1D9"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF7DF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FF244F7A"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFE8F1FF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF7DF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FF244F7A"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFE5F4F0"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF7DF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFFFFF"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FFFFF7DE"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
-      <s:patternFill patternType="solid">
-        <s:fgColor rgb="FF244F7A"/>
-      </s:patternFill>
-    </s:fill>
-    <s:fill>
+    <s:fill xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:patternFill patternType="solid">
         <s:fgColor rgb="FFF6F8FA"/>
       </s:patternFill>
     </s:fill>
-  </s:fills>
-  <s:borders count="7">
-    <s:border>
-      <s:left/>
-      <s:right/>
-      <s:top/>
-      <s:bottom/>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
-      <s:left/>
-      <s:right style="thin">
-        <s:color rgb="FFFFFFFF"/>
-      </s:right>
-      <s:top/>
-      <s:bottom/>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
-      <s:left style="thin">
-        <s:color rgb="FFFFFFFF"/>
-      </s:left>
-      <s:right style="thin">
-        <s:color rgb="FFFFFFFF"/>
-      </s:right>
-      <s:top/>
-      <s:bottom/>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
-      <s:left style="thin">
-        <s:color rgb="FFFFFFFF"/>
-      </s:left>
-      <s:right/>
-      <s:top/>
-      <s:bottom/>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
-      <s:left/>
-      <s:right/>
-      <s:top/>
-      <s:bottom style="thin">
-        <s:color rgb="FFD8E2EB"/>
-      </s:bottom>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
-      <s:left/>
-      <s:right/>
-      <s:top style="thin">
-        <s:color rgb="FFD8E2EB"/>
-      </s:top>
-      <s:bottom style="thin">
-        <s:color rgb="FFD8E2EB"/>
-      </s:bottom>
-      <s:diagonal/>
-    </s:border>
-    <s:border>
+  </fills>
+  <borders count="7">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD8E2EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD8E2EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD8E2EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <s:border xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:left/>
       <s:right/>
       <s:top style="medium">
@@ -1265,332 +1265,332 @@
       </s:bottom>
       <s:diagonal/>
     </s:border>
-  </s:borders>
-  <s:cellStyleXfs count="2">
-    <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <s:xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-  </s:cellStyleXfs>
-  <s:cellXfs count="85">
-    <s:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+  </borders>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="85">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <s:alignment vertical="top" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <s:alignment vertical="top"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <s:alignment vertical="top"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <s:alignment vertical="top"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <s:alignment vertical="top"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="top" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="0"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="14" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="14" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="14" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <s:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="15" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <s:alignment vertical="center" wrapText="1"/>
+    </s:xf>
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="15" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment horizontal="center" vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="10" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="12" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <s:alignment vertical="top"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="top" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <s:xf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="11" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <s:alignment vertical="center" wrapText="1"/>
     </s:xf>
-    <s:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="0"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="14" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="14" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="14" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="16" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="15" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="18" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="15" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </s:xf>
-    <s:xf numFmtId="0" fontId="11" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <s:alignment vertical="center" wrapText="1"/>
-    </s:xf>
-  </s:cellXfs>
-  <s:cellStyles count="2">
-    <s:cellStyle name="Normal" xfId="1"/>
-    <s:cellStyle name="표준" xfId="0"/>
-  </s:cellStyles>
-  <s:dxfs count="9">
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
-      <s:font>
-        <s:b/>
-        <s:color rgb="FFA33030"/>
-      </s:font>
-      <s:fill>
-        <s:patternFill patternType="solid">
-          <s:bgColor rgb="FFFCE4E3"/>
-        </s:patternFill>
-      </s:fill>
-    </s:dxf>
-    <s:dxf>
+  </cellXfs>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFA33030"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <s:dxf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:font>
         <s:color rgb="FF9C1D24"/>
       </s:font>
@@ -1600,7 +1600,7 @@
         </s:patternFill>
       </s:fill>
     </s:dxf>
-    <s:dxf>
+    <s:dxf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:font>
         <s:color rgb="FF536B7C"/>
       </s:font>
@@ -1610,7 +1610,7 @@
         </s:patternFill>
       </s:fill>
     </s:dxf>
-    <s:dxf>
+    <s:dxf xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
       <s:font>
         <s:color rgb="FF1C344B"/>
       </s:font>
@@ -1620,8 +1620,17 @@
         </s:patternFill>
       </s:fill>
     </s:dxf>
-  </s:dxfs>
-</s:styleSheet>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>